<commit_message>
Fix issues #22 and #23
</commit_message>
<xml_diff>
--- a/Assets/Development/TestFiles/NamedRanges.xlsx
+++ b/Assets/Development/TestFiles/NamedRanges.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\APLProjects\XL2APL\Assets\Development\TestFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EADE2619-09D7-4748-BD9D-F3BD1E0DC9EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C86F3CF7-630C-4740-802E-8CF828905659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-9290" yWindow="-21710" windowWidth="38620" windowHeight="21220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14660" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Name With Spaces" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="LocalScopeRange" localSheetId="0">Sheet1!$J$17:$L$19</definedName>
@@ -25,6 +26,8 @@
     <definedName name="MyRange4">Sheet2!$E$11:$G$11</definedName>
     <definedName name="NotaRange">"Hello world"</definedName>
     <definedName name="PI">Sheet1!$K$6</definedName>
+    <definedName name="SpaceWBScope">'Name With Spaces'!$C$4:$E$5</definedName>
+    <definedName name="SpaceWSScope" localSheetId="2">'Name With Spaces'!$D$11:$E$12</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="38">
   <si>
     <t>a</t>
   </si>
@@ -693,4 +696,52 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE297821-80D1-4290-B18D-82F4FA401239}">
+  <dimension ref="C4:E12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="4" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="C4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>